<commit_message>
Cleanup: Removed old frontend and Kaggle scripts, updated extension and backend data
</commit_message>
<xml_diff>
--- a/backend/data/custom_badwords_dataset.xlsx
+++ b/backend/data/custom_badwords_dataset.xlsx
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>dengutunnam</t>
+          <t>nee sister</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -455,7 +455,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>brother fucker</t>
+          <t>yerri</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -467,7 +467,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>tudumu</t>
+          <t>scoundrel</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -479,7 +479,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>musali</t>
+          <t>creampie</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -491,7 +491,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>🧪</t>
+          <t>thikka</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -503,7 +503,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ne ayya</t>
+          <t>paniki malina</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -515,7 +515,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>fucker</t>
+          <t>worst fellow</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -527,7 +527,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>🪲</t>
+          <t>howle</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -539,7 +539,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>🔫</t>
+          <t>pook</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -551,7 +551,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>spit</t>
+          <t>puku kodaka</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -563,7 +563,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>jule</t>
+          <t>puku</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -575,7 +575,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>noru dengutanu</t>
+          <t>nee yabba</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -587,7 +587,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>🩳</t>
+          <t>noru munda</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -599,7 +599,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>🔑</t>
+          <t>📸</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -611,7 +611,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>nee parents</t>
+          <t>coolie gadu</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -623,7 +623,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>guddalo</t>
+          <t>assault</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>modda kodaka</t>
+          <t>get lost</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>dengutunnai</t>
+          <t>nee amma</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -659,7 +659,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>gudda erri</t>
+          <t>dengey ra</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -671,7 +671,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>gudda picchi</t>
+          <t>puku erri</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -683,7 +683,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>moddalo petti</t>
+          <t>🌭</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -695,7 +695,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>☢️</t>
+          <t>basthi gadu</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -707,7 +707,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>lavadalo</t>
+          <t>nee intlo</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -719,7 +719,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>lavada lanja</t>
+          <t>🐒</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -743,7 +743,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>gutter gadu</t>
+          <t>dengutav</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>howla</t>
+          <t>🐷</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>nee family</t>
+          <t>neeku enduku</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -779,7 +779,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>humiliate</t>
+          <t>🤡</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -791,7 +791,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>nee inti valu</t>
+          <t>toilet gadu</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -803,7 +803,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>denginam</t>
+          <t>slum</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -815,7 +815,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>notlo petti dengutanu</t>
+          <t>💢</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>gajulatho</t>
+          <t>bull</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -839,7 +839,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>musuko</t>
+          <t>bloody fool</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -851,7 +851,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ne yamma</t>
+          <t>🚨</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -863,7 +863,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>chatta</t>
+          <t>dirty fellow</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -875,7 +875,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>sannasi</t>
+          <t>taagubothu</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -887,7 +887,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>lavada ra</t>
+          <t>what a loser</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -899,7 +899,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>sollu gadu</t>
+          <t>vagina</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -911,7 +911,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>dengestam</t>
+          <t>gudda lanja</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -923,7 +923,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>mentalo</t>
+          <t>nipple</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -935,7 +935,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>pukulo petti dengutanu</t>
+          <t>noru erri</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -947,7 +947,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>daridrya</t>
+          <t>dengai</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -959,7 +959,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>useless fellow</t>
+          <t>bokka donga</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -971,7 +971,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>erri na kodaka</t>
+          <t>thupuk</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -983,7 +983,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>donga</t>
+          <t>dengutadu</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>lavada</t>
+          <t>you're disgusting</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1007,7 +1007,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>🐄</t>
+          <t>modda lo</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1019,7 +1019,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>luccha</t>
+          <t>💦</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1031,7 +1031,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>🐸</t>
+          <t>dengey</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1043,7 +1043,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>auto gadu</t>
+          <t>gudda waste</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1055,7 +1055,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>get lost</t>
+          <t>🍌</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1067,7 +1067,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>🦠</t>
+          <t>🥵</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1079,7 +1079,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>bewars</t>
+          <t>dengipoyina</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1091,7 +1091,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>modda picchi</t>
+          <t>lavadalo petti dengutanu</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1103,7 +1103,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>noru musuko</t>
+          <t>🐀</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1115,7 +1115,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>witch</t>
+          <t>auto gadu</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1127,7 +1127,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>vagina</t>
+          <t>modda</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1139,7 +1139,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>snake</t>
+          <t>🩺</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1151,7 +1151,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>vadhura</t>
+          <t>moddalo</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1163,7 +1163,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>dengam</t>
+          <t>lavada donga</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1175,7 +1175,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>basthi gadu</t>
+          <t>dengesam</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>nee brother</t>
+          <t>muck</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1199,7 +1199,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ox</t>
+          <t>tagubothu</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1211,7 +1211,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>labor na kodaka</t>
+          <t>🛡️</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1223,7 +1223,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>tits</t>
+          <t>guddalo petti</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1235,7 +1235,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>item</t>
+          <t>dengindi</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1247,7 +1247,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>dongana kodaka</t>
+          <t>madda</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1259,7 +1259,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>卐</t>
+          <t>😾</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1271,7 +1271,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>bokka le</t>
+          <t>denginadi</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1283,7 +1283,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>brute</t>
+          <t>💊</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1295,7 +1295,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>modda waste</t>
+          <t>nee family</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>pooku</t>
+          <t>gajulatho</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -1319,7 +1319,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>lizard</t>
+          <t>chatta</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -1331,7 +1331,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>bokka munda</t>
+          <t>sperm</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -1343,7 +1343,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>erripappa</t>
+          <t>julayi</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -1355,7 +1355,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>lavada picchi</t>
+          <t>pukulo petti</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>guddalo dengutanu</t>
+          <t>whore</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -1379,7 +1379,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>nee mother</t>
+          <t>bokkalo petti dengutanu</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -1391,7 +1391,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>dunnapothu</t>
+          <t>lavadalo</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -1403,7 +1403,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>nasty</t>
+          <t>motherfucker</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -1415,7 +1415,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>denganu</t>
+          <t>fraud gadu</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -1427,7 +1427,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>lanjakodaka</t>
+          <t>🐄</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -1439,7 +1439,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>boobs</t>
+          <t>chetha</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -1451,7 +1451,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>pichi lanjakodaka</t>
+          <t>dengesadu</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -1463,7 +1463,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>waste fellow</t>
+          <t>nobody asked</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -1475,7 +1475,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>🪃</t>
+          <t>hook gadu</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -1487,7 +1487,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>bastard</t>
+          <t>close your mouth</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -1499,7 +1499,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>rowdy</t>
+          <t>traffic fellow</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -1511,7 +1511,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>parasite</t>
+          <t>musali</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -1523,7 +1523,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>puk</t>
+          <t>howla</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -1535,7 +1535,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>gudda dengutanu</t>
+          <t>worst gadu</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>howle</t>
+          <t>rakshasi</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -1559,7 +1559,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>nee ayya</t>
+          <t>road gadu</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -1571,7 +1571,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>signal gadu</t>
+          <t>third class</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>gudda lanja</t>
+          <t>daridrya</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -1595,7 +1595,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>dengey</t>
+          <t>vermin</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -1607,7 +1607,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>😾</t>
+          <t>addamina</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -1619,7 +1619,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>idiot</t>
+          <t>dengestav</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -1631,7 +1631,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>pendu</t>
+          <t>pichi lanjakodaka</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -1643,7 +1643,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>picchi</t>
+          <t>pichi pulka</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -1655,7 +1655,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>guddalo petti</t>
+          <t>bokka dengutanu</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>dengutunna</t>
+          <t>waste fellow</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -1679,7 +1679,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>dengesanu</t>
+          <t>sulli</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -1691,7 +1691,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>sister fucker</t>
+          <t>dongana kodaka</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -1703,7 +1703,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>taagubothu</t>
+          <t>💋</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -1715,7 +1715,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>bokka lo</t>
+          <t>nee husband</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>pakodi</t>
+          <t>🪳</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -1739,7 +1739,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>👅</t>
+          <t>🪲</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -1751,7 +1751,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>yadava</t>
+          <t>guddalo dengutanu</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -1763,7 +1763,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>bazar dana</t>
+          <t>low class</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -1775,7 +1775,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>bitch</t>
+          <t>suicide</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -1787,7 +1787,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>bokka waste</t>
+          <t>lavada lo</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -1799,7 +1799,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>uncivilized</t>
+          <t>dengutunnam</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -1811,7 +1811,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>🗡️</t>
+          <t>ranku munda</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -1823,7 +1823,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>shikandi</t>
+          <t>durmargudu</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -1835,7 +1835,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>dengesam</t>
+          <t>dengutunnadu</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -1847,7 +1847,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>noru picchi</t>
+          <t>cunt</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -1859,7 +1859,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>dengutunnav</t>
+          <t>screwed</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -1871,7 +1871,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>semen</t>
+          <t>you are an idiot</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -1883,7 +1883,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>💣</t>
+          <t>nee fuku</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -1895,7 +1895,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>you are an idiot</t>
+          <t>dengichuko</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -1907,7 +1907,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>dengutadu</t>
+          <t>pukulo petti dengutanu</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -1919,7 +1919,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>nobody asked for your opinion</t>
+          <t>bocchu</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -1931,7 +1931,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>bokkalo dengutanu</t>
+          <t>violate</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -1943,7 +1943,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>卍</t>
+          <t>vulture</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -1955,7 +1955,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>puku dengutanu</t>
+          <t>🐸</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -1967,7 +1967,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>vedhava</t>
+          <t>💀</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -1979,7 +1979,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>mule</t>
+          <t>pandi</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -1991,7 +1991,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>dengutunnadu</t>
+          <t>🐛</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -2003,7 +2003,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>you're annoying</t>
+          <t>ne yamma</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -2015,7 +2015,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>gudda</t>
+          <t>scum</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -2027,7 +2027,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>dengav</t>
+          <t>monkey</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -2039,7 +2039,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>you are stupid</t>
+          <t>psycho</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -2051,7 +2051,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>sollu</t>
+          <t>erri pushpam</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -2063,7 +2063,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>🪳</t>
+          <t>puku picchi</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -2075,7 +2075,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>🖕🏼</t>
+          <t>squirt</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -2087,7 +2087,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>🤮</t>
+          <t>gudda kodaka</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -2099,7 +2099,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>you're trash</t>
+          <t>idiot</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -2111,7 +2111,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>denginaru</t>
+          <t>puku waste</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -2123,7 +2123,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>donga munda</t>
+          <t>parasite</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -2135,7 +2135,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>🧨</t>
+          <t>🤙</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -2147,7 +2147,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>fuck</t>
+          <t>vadhura</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -2159,7 +2159,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>nee father</t>
+          <t>lavada le</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -2171,7 +2171,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>🍌</t>
+          <t>tirugubothu</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -2183,7 +2183,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>trash</t>
+          <t>sadist</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -2195,7 +2195,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>kys</t>
+          <t>lavada waste</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -2207,7 +2207,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>dengutanu</t>
+          <t>thirugubothu</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -2219,7 +2219,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>chatta na kodaka</t>
+          <t>☠️</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -2231,7 +2231,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>💉</t>
+          <t>jackass</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -2243,7 +2243,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ranku munda</t>
+          <t>🦠</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -2255,7 +2255,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>mundamopi</t>
+          <t>notlo</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -2267,7 +2267,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>420</t>
+          <t>boobs</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -2279,7 +2279,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>🍑</t>
+          <t>pukulo dengutanu</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -2291,7 +2291,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>madda</t>
+          <t>bokka lo</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -2303,7 +2303,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>julayi</t>
+          <t>🤛</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -2315,7 +2315,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>humped</t>
+          <t>🪓</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -2327,7 +2327,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>yedava</t>
+          <t>musuko</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -2339,7 +2339,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>☠️</t>
+          <t>modda ra</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -2351,7 +2351,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>bokka donga</t>
+          <t>nee ayya</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -2363,7 +2363,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>🤙</t>
+          <t>modda lanja</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -2375,7 +2375,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>chapri</t>
+          <t>nee abba</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -2387,7 +2387,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>bokka lanja</t>
+          <t>filth</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -2399,7 +2399,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>pichi pulka</t>
+          <t>noru le</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -2411,7 +2411,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>buffalo</t>
+          <t>moddalo petti dengutanu</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -2423,7 +2423,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>go to hell</t>
+          <t>bitch</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -2435,7 +2435,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>lavada donga</t>
+          <t>💩</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -2447,7 +2447,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>chavata</t>
+          <t>fucking</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -2459,7 +2459,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>siggu leni</t>
+          <t>harass</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -2471,7 +2471,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>suicide</t>
+          <t>waste gadu</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -2483,7 +2483,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>erri puku</t>
+          <t>🖕🏼</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -2495,7 +2495,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>gudda donga</t>
+          <t>modda erri</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -2507,7 +2507,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>slum</t>
+          <t>🪃</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -2519,7 +2519,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>dengey ra</t>
+          <t>noru muyyi</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -2531,7 +2531,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>rakshasi</t>
+          <t>noru dengutanu</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -2543,7 +2543,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>modda</t>
+          <t>dengutunnav</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -2555,7 +2555,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>notlo petti</t>
+          <t>labor gadu</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -2567,7 +2567,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>whore</t>
+          <t>lavada lanja</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -2579,7 +2579,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>monkey</t>
+          <t>🏹</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -2591,7 +2591,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>noru lanja</t>
+          <t>witch</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -2603,7 +2603,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>you deserve to die</t>
+          <t>strangle</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -2615,7 +2615,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>local gadu</t>
+          <t>bhadcow</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -2627,7 +2627,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>waste gadu</t>
+          <t>slut</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -2639,7 +2639,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>basthi fellow</t>
+          <t>🖕🏿</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -2651,7 +2651,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>3rd class</t>
+          <t>i hate you</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -2663,7 +2663,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>lavada waste</t>
+          <t>vedava</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -2675,7 +2675,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>worst gadu</t>
+          <t>picchi</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -2687,7 +2687,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>lavada dengutanu</t>
+          <t>puk</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -2699,7 +2699,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>🚨</t>
+          <t>basthi fellow</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -2711,7 +2711,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>avalanja</t>
+          <t>dengesai</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -2723,7 +2723,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>🔞</t>
+          <t>kojja</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -2735,7 +2735,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>toilet gadu</t>
+          <t>lavada picchi</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -2747,7 +2747,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>slut</t>
+          <t>🍒</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -2759,7 +2759,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>stupid</t>
+          <t>you're annoying</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -2771,7 +2771,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>📸</t>
+          <t>noru picchi</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -2783,7 +2783,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>denginchukunna</t>
+          <t>kys</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -2795,7 +2795,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>☣️</t>
+          <t>addamina panulu</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -2807,7 +2807,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>dengesav</t>
+          <t>fucked</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -2819,7 +2819,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>noru le</t>
+          <t>you're ugly</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -2831,7 +2831,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>close your mouth</t>
+          <t>puku le</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -2843,7 +2843,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>garbage gadu</t>
+          <t>suffocate</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -2855,7 +2855,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>noru erri</t>
+          <t>useless fellow</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -2867,7 +2867,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>shut up</t>
+          <t>lavada kodaka</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -2879,7 +2879,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>modda donga</t>
+          <t>😡</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -2891,7 +2891,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>bokka ra</t>
+          <t>cheap fellow</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -2903,7 +2903,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>dengali</t>
+          <t>penis</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -2915,7 +2915,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>fucked</t>
+          <t>basthi</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -2927,7 +2927,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>nee amma</t>
+          <t>👿</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -2939,7 +2939,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>addamina</t>
+          <t>bokka erri</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -2951,7 +2951,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>bloody fool</t>
+          <t>modda le</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -2963,7 +2963,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>🪓</t>
+          <t>leech</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -2975,7 +2975,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>👿</t>
+          <t>🤢</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -2987,7 +2987,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>⚰️</t>
+          <t>savage</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -2999,7 +2999,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>puku kodaka</t>
+          <t>dengestai</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -3011,7 +3011,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>harass</t>
+          <t>loafer</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -3023,7 +3023,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>dirty fellow</t>
+          <t>nee mother</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -3035,7 +3035,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>donga na kodaka</t>
+          <t>stupid ga unnav</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -3047,7 +3047,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>thupuk</t>
+          <t>gudda le</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -3059,7 +3059,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>dengestadu</t>
+          <t>☢️</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -3071,7 +3071,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>gudda waste</t>
+          <t>erri puku</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -3083,7 +3083,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>nobody asked</t>
+          <t>coolie</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -3095,7 +3095,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>jaffa</t>
+          <t>rakshasuda</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -3107,7 +3107,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>prostitute</t>
+          <t>kukka</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -3119,7 +3119,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>modda dengutanu</t>
+          <t>🍫</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -3131,7 +3131,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>🤬</t>
+          <t>dick</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -3143,7 +3143,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>denginadu</t>
+          <t>konda erri</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -3155,7 +3155,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>slap</t>
+          <t>gaadida</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>dengestadi</t>
+          <t>neeku enduku ra</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -3179,7 +3179,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>errihook</t>
+          <t>dengesanu</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -3191,7 +3191,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>kothi</t>
+          <t>ni bondha</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -3203,7 +3203,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>scoundrel</t>
+          <t>bokulo</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -3215,7 +3215,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>🛏️</t>
+          <t>sannasi</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -3227,7 +3227,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>father fucker</t>
+          <t>lavada munda</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -3239,7 +3239,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>dengadu</t>
+          <t>noru musuko</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -3251,7 +3251,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>bazaru munda</t>
+          <t>fuck</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -3263,7 +3263,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>pavement fellow</t>
+          <t>puku lanja</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -3275,7 +3275,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>🩺</t>
+          <t>loser</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -3287,7 +3287,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>bull</t>
+          <t>manhole gadu</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -3299,7 +3299,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>ni bondha</t>
+          <t>road meeda tige dana</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -3311,7 +3311,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>🙊</t>
+          <t>bokka munda</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -3323,7 +3323,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>thikka</t>
+          <t>erri na kodaka</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -3335,7 +3335,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>lajja</t>
+          <t>molest</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -3347,7 +3347,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>spunk</t>
+          <t>chapri gadu</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -3359,7 +3359,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>fake gadu</t>
+          <t>ne ayya</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -3371,7 +3371,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>bokka dengutanu</t>
+          <t>puku dengutanu</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -3383,7 +3383,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>💊</t>
+          <t>modda picchi</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -3395,7 +3395,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>noru kodaka</t>
+          <t>sewer gadu</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -3407,7 +3407,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>modda lanja</t>
+          <t>odiyamma</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -3419,7 +3419,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>kill yourself</t>
+          <t>dengesav</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -3431,7 +3431,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>nee yabba</t>
+          <t>denganu</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -3443,7 +3443,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>kojja</t>
+          <t>puku donga</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -3455,7 +3455,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>suffocate</t>
+          <t>🖕🏽</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -3467,7 +3467,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>hook gadu</t>
+          <t>cock</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -3479,7 +3479,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>vulture</t>
+          <t>vedhava</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -3491,7 +3491,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>what a loser</t>
+          <t>humiliate</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -3503,7 +3503,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>yerri</t>
+          <t>gadida</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -3515,7 +3515,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>dick</t>
+          <t>noru kodaka</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -3527,7 +3527,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>footpath gadu</t>
+          <t>dengichukuntunna</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -3539,7 +3539,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>maggot</t>
+          <t>卐</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -3551,7 +3551,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>konda erri</t>
+          <t>moddalo dengutanu</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -3563,7 +3563,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>🖕🏿</t>
+          <t>you're trash</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -3575,7 +3575,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>bokkalo petti dengutanu</t>
+          <t>rowdy</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -3587,7 +3587,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>dengina</t>
+          <t>modda munda</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -3599,7 +3599,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>kukka</t>
+          <t>nasty</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -3611,7 +3611,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>sulliga</t>
+          <t>jule</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -3623,7 +3623,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>dengey le</t>
+          <t>gudda dengutanu</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -3635,7 +3635,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>bokulo</t>
+          <t>go to hell</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -3647,7 +3647,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>fraud gadu</t>
+          <t>dengipotha</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -3659,7 +3659,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>dengipoyina</t>
+          <t>gutter gadu</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -3671,7 +3671,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>lavada le</t>
+          <t>dengu</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -3683,7 +3683,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>motherfucker</t>
+          <t>pavement fellow</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -3695,7 +3695,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>dengutadi</t>
+          <t>bokka ra</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -3707,7 +3707,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>🐮</t>
+          <t>fucker</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -3719,7 +3719,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>choke</t>
+          <t>dengipoya</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -3731,7 +3731,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>horny</t>
+          <t>poramboku</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -3743,7 +3743,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>nee wife</t>
+          <t>420</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
@@ -3755,7 +3755,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>dengutai</t>
+          <t>⚠️</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -3767,7 +3767,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>you're ugly</t>
+          <t>rape</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -3779,7 +3779,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>dengu</t>
+          <t>3rd class</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -3791,7 +3791,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>puku munda</t>
+          <t>riksha gadu</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -3803,7 +3803,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>loafer</t>
+          <t>denginav</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -3815,7 +3815,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>riksha gadu</t>
+          <t>gudda ra</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -3827,7 +3827,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>puku waste</t>
+          <t>sweeper gadu</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -3839,7 +3839,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>dengipoya</t>
+          <t>lavada</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -3851,7 +3851,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>gudda kodaka</t>
+          <t>notlo petti</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -3863,7 +3863,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>sani</t>
+          <t>dengav</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -3875,7 +3875,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>noru munda</t>
+          <t>chettana kodaka</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -3887,7 +3887,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>modda lo</t>
+          <t>mule</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -3899,7 +3899,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>dengutunnadi</t>
+          <t>pooku</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -3911,7 +3911,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>dengai</t>
+          <t>卍</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -3923,7 +3923,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>rascal</t>
+          <t>bewarsi</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -3935,7 +3935,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>chettana kodaka</t>
+          <t>💉</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -3947,7 +3947,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>sperm</t>
+          <t>uncivilized</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -3959,7 +3959,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>lanja</t>
+          <t>bokkalo dengutanu</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -3971,7 +3971,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>💩</t>
+          <t>item</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -3983,7 +3983,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>🖕🏽</t>
+          <t>slap</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
@@ -3995,7 +3995,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>coolie</t>
+          <t>you deserve to die</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
@@ -4007,7 +4007,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>dengindi</t>
+          <t>dengutunnanu</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -4019,7 +4019,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>gudda munda</t>
+          <t>shagged</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -4031,7 +4031,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>nipple</t>
+          <t>👙</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -4043,7 +4043,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>dengesta</t>
+          <t>gudda munda</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -4055,7 +4055,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>chetta</t>
+          <t>kothi vedhava</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -4067,7 +4067,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>⚠️</t>
+          <t>nee brother</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -4079,7 +4079,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>nee intlo</t>
+          <t>fake gadu</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -4091,7 +4091,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>🥵</t>
+          <t>dengaru</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -4103,7 +4103,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>denginadi</t>
+          <t>jaffa</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -4115,7 +4115,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>odiyamma</t>
+          <t>maggot</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -4127,7 +4127,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>munda</t>
+          <t>lajja</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -4139,7 +4139,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>🤡</t>
+          <t>modda dengutanu</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
@@ -4151,7 +4151,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>dustbin gadu</t>
+          <t>spit</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -4163,7 +4163,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>ne kamma</t>
+          <t>pichi na kodaka</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -4175,7 +4175,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>🐀</t>
+          <t>denginadu</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -4187,7 +4187,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>denginai</t>
+          <t>dengutha</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -4199,7 +4199,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>🍒</t>
+          <t>denginai</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -4211,7 +4211,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>low class fellow</t>
+          <t>avalanja</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
@@ -4223,7 +4223,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>road fellow</t>
+          <t>nee father</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
@@ -4235,7 +4235,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>strangle</t>
+          <t>chapri</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>4th class</t>
+          <t>shut up</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -4259,7 +4259,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>modda ra</t>
+          <t>lavadalo dengutanu</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -4271,7 +4271,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>you're worthless</t>
+          <t>footpath gadu</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -4283,7 +4283,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>traffic fellow</t>
+          <t>waste body</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
@@ -4295,7 +4295,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>dengaru</t>
+          <t>dengestadu</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
@@ -4307,7 +4307,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>erri pushpam</t>
+          <t>bastard</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
@@ -4319,7 +4319,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>i hate you</t>
+          <t>🍑</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
@@ -4331,7 +4331,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>addamina panulu</t>
+          <t>👊</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
@@ -4343,7 +4343,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>puku lanja</t>
+          <t>musukoni kurcho</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -4355,7 +4355,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>you're so dumb</t>
+          <t>you are stupid</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -4367,7 +4367,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>💀</t>
+          <t>pest</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -4379,7 +4379,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>pussy</t>
+          <t>tudumu</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -4391,7 +4391,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>dengesadi</t>
+          <t>nee inti valu</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -4403,7 +4403,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>moddalo</t>
+          <t>humped</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -4415,7 +4415,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>🔪</t>
+          <t>stupid</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -4427,7 +4427,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>🩸</t>
+          <t>lanja</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -4439,7 +4439,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>guddalo petti dengutanu</t>
+          <t>drain gadu</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -4451,7 +4451,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>kojja na kodaka</t>
+          <t>gudda</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -4463,7 +4463,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>🍆</t>
+          <t>bhadkaw</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -4475,7 +4475,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>pichi na kodaka</t>
+          <t>puku munda</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -4487,7 +4487,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>fucking</t>
+          <t>kothi</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -4499,7 +4499,7 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>notlo dengutanu</t>
+          <t>slum fellow</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
@@ -4511,7 +4511,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>bhadcow</t>
+          <t>lavada dengutanu</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -4523,7 +4523,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>solu</t>
+          <t>sollu gadu</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
@@ -4535,7 +4535,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>⚔️</t>
+          <t>notlo petti dengutanu</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
@@ -4547,7 +4547,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>🖕🏻</t>
+          <t>abuse</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
@@ -4559,7 +4559,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>abuse</t>
+          <t>noru lanja</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -4571,7 +4571,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>waste na kodaka</t>
+          <t>🤜</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -4583,7 +4583,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>thirugubothu</t>
+          <t>denginchukunna</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -4595,7 +4595,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>jackass</t>
+          <t>🖕🏻</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
@@ -4607,7 +4607,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>tirugubothu</t>
+          <t>🩸</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -4619,7 +4619,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>dengutunnaru</t>
+          <t>sulliga</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -4631,7 +4631,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>🍫</t>
+          <t>boku</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -4643,7 +4643,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>sweeper gadu</t>
+          <t>badcow</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
@@ -4655,7 +4655,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>degrade</t>
+          <t>luccha</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
@@ -4667,7 +4667,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>lavada erri</t>
+          <t>🩲</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
@@ -4679,7 +4679,7 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>slum fellow</t>
+          <t>dengutunnaru</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
@@ -4691,7 +4691,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>lavada lo</t>
+          <t>☣️</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
@@ -4703,7 +4703,7 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>🖕</t>
+          <t>dustbin gadu</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
@@ -4715,7 +4715,7 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>vermin</t>
+          <t>lanjakodaka</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
@@ -4727,7 +4727,7 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>this is garbage</t>
+          <t>🔪</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
@@ -4739,7 +4739,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>lavadalo dengutanu</t>
+          <t>dengutanu</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -4751,7 +4751,7 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>bokka kodaka</t>
+          <t>🗡️</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
@@ -4763,7 +4763,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>penis</t>
+          <t>gudda lo</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -4775,7 +4775,7 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>lavada munda</t>
+          <t>dengadu</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
@@ -4787,7 +4787,7 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>street fellow</t>
+          <t>solu</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
@@ -4799,7 +4799,7 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>👊</t>
+          <t>snake</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
@@ -4811,7 +4811,7 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>🐷</t>
+          <t>guddalo</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
@@ -4823,7 +4823,7 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>lavadalo petti dengutanu</t>
+          <t>lavada erri</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
@@ -4835,7 +4835,7 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>shagged</t>
+          <t>nee wife</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
@@ -4847,7 +4847,7 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>puku donga</t>
+          <t>you're worthless</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
@@ -4859,7 +4859,7 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>pandi</t>
+          <t>dengutam</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
@@ -4871,7 +4871,7 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>leech</t>
+          <t>puku lo</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
@@ -4883,7 +4883,7 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>molest</t>
+          <t>dengutunnadi</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
@@ -4895,7 +4895,7 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>barbarian</t>
+          <t>buffalo</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
@@ -4907,7 +4907,7 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>denginav</t>
+          <t>dengali</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
@@ -4919,7 +4919,7 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>noru ra</t>
+          <t>brother fucker</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
@@ -4931,7 +4931,7 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>shit</t>
+          <t>waste na kodaka</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
@@ -4943,7 +4943,7 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>moddalo dengutanu</t>
+          <t>semen</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
@@ -4955,7 +4955,7 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>🤢</t>
+          <t>dengutai</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
@@ -4967,7 +4967,7 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>🐒</t>
+          <t>🛏️</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
@@ -4979,7 +4979,7 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>pulka</t>
+          <t>puku ra</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
@@ -4991,7 +4991,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>🤏</t>
+          <t>bewars</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
@@ -5003,7 +5003,7 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>nee husband</t>
+          <t>barbarian</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
@@ -5015,7 +5015,7 @@
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>moddalo petti dengutanu</t>
+          <t>bokka waste</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
@@ -5027,7 +5027,7 @@
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>dengesadu</t>
+          <t>rascal</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
@@ -5039,7 +5039,7 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>labor gadu</t>
+          <t>you're so dumb</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
@@ -5051,7 +5051,7 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>dengestav</t>
+          <t>🖕</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
@@ -5063,7 +5063,7 @@
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>pest</t>
+          <t>👅</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
@@ -5075,7 +5075,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>you're pathetic</t>
+          <t>pakodi</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
@@ -5087,7 +5087,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>bewarsi</t>
+          <t>🌮</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
@@ -5099,7 +5099,7 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>garbage</t>
+          <t>⚰️</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
@@ -5111,7 +5111,7 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>you're disgusting</t>
+          <t>you're pathetic</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
@@ -5123,7 +5123,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>grime</t>
+          <t>dengesadi</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -5135,7 +5135,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>i will find you</t>
+          <t>🔫</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>creampie</t>
+          <t>pulka</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
@@ -5159,7 +5159,7 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>notlo</t>
+          <t>street fellow</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
@@ -5171,7 +5171,7 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>cock</t>
+          <t>sister fucker</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
@@ -5183,7 +5183,7 @@
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>🛡️</t>
+          <t>🤬</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
@@ -5195,7 +5195,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>🌮</t>
+          <t>noru ra</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
@@ -5207,7 +5207,7 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>boku</t>
+          <t>🙊</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
@@ -5219,7 +5219,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>dengichukuntunna</t>
+          <t>ne kamma</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
@@ -5231,7 +5231,7 @@
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>poramboku</t>
+          <t>nobody likes you</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
@@ -5243,7 +5243,7 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>modda munda</t>
+          <t>dengutaru</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
@@ -5255,7 +5255,7 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>neeku enduku</t>
+          <t>yedava</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
@@ -5267,7 +5267,7 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>road meeda tige dana</t>
+          <t>labor na kodaka</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
@@ -5279,7 +5279,7 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>dengutaru</t>
+          <t>🔞</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
@@ -5291,7 +5291,7 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>🪦</t>
+          <t>sollu</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
@@ -5303,7 +5303,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>lavada kodaka</t>
+          <t>lizard</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -5315,7 +5315,7 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>basthi</t>
+          <t>siggu leni</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
@@ -5327,7 +5327,7 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>stupid ga unnav</t>
+          <t>dunnapothu</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
@@ -5339,7 +5339,7 @@
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>buffoon</t>
+          <t>road fellow</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
@@ -5351,7 +5351,7 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>👙</t>
+          <t>dengam</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
@@ -5363,7 +5363,7 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>💋</t>
+          <t>horny</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
@@ -5375,7 +5375,7 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>slime</t>
+          <t>lavada ra</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>🐛</t>
+          <t>gudda erri</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
@@ -5399,7 +5399,7 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>pook</t>
+          <t>dengina</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
@@ -5411,7 +5411,7 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>🐖</t>
+          <t>🔑</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
@@ -5423,7 +5423,7 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>chapri gadu</t>
+          <t>bokka picchi</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
@@ -5435,7 +5435,7 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>bocchu</t>
+          <t>degrade</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
@@ -5447,7 +5447,7 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>bhadkaw</t>
+          <t>nee parents</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
@@ -5459,7 +5459,7 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>dengutunnanu</t>
+          <t>dengutadi</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
@@ -5471,7 +5471,7 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>waste body</t>
+          <t>kojja na kodaka</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
@@ -5483,7 +5483,7 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>dengutav</t>
+          <t>chetta</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
@@ -5495,7 +5495,7 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>dengutam</t>
+          <t>sani</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
@@ -5507,7 +5507,7 @@
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>hijra</t>
+          <t>🩳</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
@@ -5519,7 +5519,7 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>rakshasuda</t>
+          <t>i will find you</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
@@ -5531,7 +5531,7 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>🖕🏾</t>
+          <t>low class fellow</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
@@ -5543,7 +5543,7 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>gaadida</t>
+          <t>dengesaru</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
@@ -5555,7 +5555,7 @@
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>💢</t>
+          <t>noru donga</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
@@ -5567,7 +5567,7 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>gadida</t>
+          <t>spunk</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
@@ -5579,7 +5579,7 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>erri</t>
+          <t>dengesta</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
@@ -5591,7 +5591,7 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>dengesaru</t>
+          <t>garbage gadu</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
@@ -5603,7 +5603,7 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>noru donga</t>
+          <t>donga</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
@@ -5615,7 +5615,7 @@
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>cunt</t>
+          <t>modda kodaka</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
@@ -5627,7 +5627,7 @@
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>dengestaru</t>
+          <t>dengutunna</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
@@ -5639,7 +5639,7 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>💦</t>
+          <t>moddalo petti</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
@@ -5651,7 +5651,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>dengutha</t>
+          <t>🪦</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -5663,7 +5663,7 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>filth</t>
+          <t>shikandi</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
@@ -5675,7 +5675,7 @@
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>screwed</t>
+          <t>gudda picchi</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
@@ -5687,7 +5687,7 @@
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>puku le</t>
+          <t>trash</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
@@ -5699,7 +5699,7 @@
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>pukulo dengutanu</t>
+          <t>shit</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
@@ -5711,7 +5711,7 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>nee fuku</t>
+          <t>asshole</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
@@ -5723,7 +5723,7 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>badcow</t>
+          <t>notlo dengutanu</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
@@ -5735,7 +5735,7 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>durmargudu</t>
+          <t>pendu</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
@@ -5747,7 +5747,7 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>neeku enduku ra</t>
+          <t>erri</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
@@ -5759,7 +5759,7 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>modda erri</t>
+          <t>bazar dana</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
@@ -5771,7 +5771,7 @@
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>asshole</t>
+          <t>💣</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
@@ -5783,7 +5783,7 @@
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>cheap fellow</t>
+          <t>yadava</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
@@ -5795,7 +5795,7 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>dengipotha</t>
+          <t>bazaru munda</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
@@ -5807,7 +5807,7 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>jizz</t>
+          <t>dengestaru</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
@@ -5819,7 +5819,7 @@
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>gudda ra</t>
+          <t>choke</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
@@ -5831,7 +5831,7 @@
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>puku</t>
+          <t>dengutunnai</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
@@ -5843,7 +5843,7 @@
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>musukoni kurcho</t>
+          <t>bokka le</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
@@ -5855,7 +5855,7 @@
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>gudda le</t>
+          <t>munda</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
@@ -5867,7 +5867,7 @@
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>gudda lo</t>
+          <t>tits</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
@@ -5879,7 +5879,7 @@
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>drain gadu</t>
+          <t>erripappa</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
@@ -5891,7 +5891,7 @@
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>psycho</t>
+          <t>kill yourself</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
@@ -5903,7 +5903,7 @@
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>sadist</t>
+          <t>jizz</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
@@ -5915,7 +5915,7 @@
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>violate</t>
+          <t>🧪</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
@@ -5927,7 +5927,7 @@
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>pukulo petti</t>
+          <t>bokka lanja</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
@@ -5939,7 +5939,7 @@
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>😡</t>
+          <t>ox</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
@@ -5951,7 +5951,7 @@
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>puku picchi</t>
+          <t>😤</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
@@ -5963,7 +5963,7 @@
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>assault</t>
+          <t>🧨</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
@@ -5975,7 +5975,7 @@
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>🩲</t>
+          <t>hijra</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>muck</t>
+          <t>dengey le</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
@@ -5999,7 +5999,7 @@
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>sewer gadu</t>
+          <t>🍆</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
@@ -6011,7 +6011,7 @@
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>manhole gadu</t>
+          <t>prostitute</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
@@ -6023,7 +6023,7 @@
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>noru muyyi</t>
+          <t>buffoon</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
@@ -6035,7 +6035,7 @@
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>vedava</t>
+          <t>denginam</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
@@ -6047,7 +6047,7 @@
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>puku lo</t>
+          <t>garbage</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
@@ -6059,7 +6059,7 @@
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>lanja kodaka</t>
+          <t>🤏</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
@@ -6071,7 +6071,7 @@
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>chetha</t>
+          <t>father fucker</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
@@ -6083,7 +6083,7 @@
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>loser</t>
+          <t>dengestam</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
@@ -6095,7 +6095,7 @@
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>squirt</t>
+          <t>4th class</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
@@ -6107,7 +6107,7 @@
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>🌭</t>
+          <t>dengestadi</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
@@ -6119,7 +6119,7 @@
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>puku erri</t>
+          <t>bokka kodaka</t>
         </is>
       </c>
       <c r="B475" t="inlineStr">
@@ -6131,7 +6131,7 @@
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>noru waste</t>
+          <t>modda waste</t>
         </is>
       </c>
       <c r="B476" t="inlineStr">
@@ -6143,7 +6143,7 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>worst fellow</t>
+          <t>ni abba</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
@@ -6155,7 +6155,7 @@
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>third class</t>
+          <t>mentalo</t>
         </is>
       </c>
       <c r="B478" t="inlineStr">
@@ -6167,7 +6167,7 @@
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>paniki malina</t>
+          <t>noru waste</t>
         </is>
       </c>
       <c r="B479" t="inlineStr">
@@ -6179,7 +6179,7 @@
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>road gadu</t>
+          <t>denginaru</t>
         </is>
       </c>
       <c r="B480" t="inlineStr">
@@ -6191,7 +6191,7 @@
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>low class</t>
+          <t>donga na kodaka</t>
         </is>
       </c>
       <c r="B481" t="inlineStr">
@@ -6203,7 +6203,7 @@
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>dengesai</t>
+          <t>donga munda</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
@@ -6215,7 +6215,7 @@
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>kothi vedhava</t>
+          <t>🤮</t>
         </is>
       </c>
       <c r="B483" t="inlineStr">
@@ -6227,7 +6227,7 @@
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>🏹</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
@@ -6239,7 +6239,7 @@
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>modda le</t>
+          <t>grime</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
@@ -6251,7 +6251,7 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>sulli</t>
+          <t>chavata</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
@@ -6263,7 +6263,7 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>tagubothu</t>
+          <t>this is garbage</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
@@ -6275,7 +6275,7 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>coolie gadu</t>
+          <t>slime</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
@@ -6287,7 +6287,7 @@
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>scum</t>
+          <t>local gadu</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
@@ -6299,7 +6299,7 @@
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>bokka erri</t>
+          <t>chatta na kodaka</t>
         </is>
       </c>
       <c r="B490" t="inlineStr">
@@ -6311,7 +6311,7 @@
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>🤛</t>
+          <t>nobody asked for your opinion</t>
         </is>
       </c>
       <c r="B491" t="inlineStr">
@@ -6323,7 +6323,7 @@
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>puku ra</t>
+          <t>🐮</t>
         </is>
       </c>
       <c r="B492" t="inlineStr">
@@ -6335,7 +6335,7 @@
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>nobody likes you</t>
+          <t>🖕🏾</t>
         </is>
       </c>
       <c r="B493" t="inlineStr">
@@ -6347,7 +6347,7 @@
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>ni abba</t>
+          <t>guddalo petti dengutanu</t>
         </is>
       </c>
       <c r="B494" t="inlineStr">
@@ -6359,7 +6359,7 @@
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>rape</t>
+          <t>pussy</t>
         </is>
       </c>
       <c r="B495" t="inlineStr">
@@ -6371,7 +6371,7 @@
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>savage</t>
+          <t>signal gadu</t>
         </is>
       </c>
       <c r="B496" t="inlineStr">
@@ -6383,7 +6383,7 @@
     <row r="497">
       <c r="A497" t="inlineStr">
         <is>
-          <t>bokka picchi</t>
+          <t>gudda donga</t>
         </is>
       </c>
       <c r="B497" t="inlineStr">
@@ -6395,7 +6395,7 @@
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>dengestai</t>
+          <t>modda donga</t>
         </is>
       </c>
       <c r="B498" t="inlineStr">
@@ -6407,7 +6407,7 @@
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>nee abba</t>
+          <t>🐖</t>
         </is>
       </c>
       <c r="B499" t="inlineStr">
@@ -6419,7 +6419,7 @@
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>dengichuko</t>
+          <t>errihook</t>
         </is>
       </c>
       <c r="B500" t="inlineStr">
@@ -6431,7 +6431,7 @@
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>nee sister</t>
+          <t>mundamopi</t>
         </is>
       </c>
       <c r="B501" t="inlineStr">
@@ -6443,7 +6443,7 @@
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>😤</t>
+          <t>lanja kodaka</t>
         </is>
       </c>
       <c r="B502" t="inlineStr">
@@ -6455,7 +6455,7 @@
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>🤜</t>
+          <t>brute</t>
         </is>
       </c>
       <c r="B503" t="inlineStr">

</xml_diff>